<commit_message>
May: intro e ajustes
</commit_message>
<xml_diff>
--- a/tabela de habitat.xlsx
+++ b/tabela de habitat.xlsx
@@ -1,27 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="tabela_final" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="tabela_final" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
-  <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="756" uniqueCount="541">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="511">
   <si>
     <t xml:space="preserve">Variable</t>
   </si>
@@ -930,96 +924,6 @@
   </si>
   <si>
     <t xml:space="preserve">Qualidade da água</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Temperatura da água (°C) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">12,9 (0-27,3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13,3 (0-27,5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12,6 (0-25,5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13,9 (0-28,5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13,5 (0-27,3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13,2 (0-26,5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13,4 (0-27,4)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13,6 (0-27,2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13,9 (0-28)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14,6 (0-29,3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16,2 (0-33,4)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14,3 (0-29,1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14,3 (0-28,9)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14,3 (0-28,6)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14,1 (0-28,2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oxigênio dissolvido (mg/L) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">4,1 (0-8,5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3,8 (0-7,8)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3,9 (0-8)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3,8 (0-8,4)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3,9 (0-7,9)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2,7 (0-6,1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3,8 (0-8,1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3,5 (0-7,5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3,1 (0-6,8)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2,6 (0-5,4)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3,5 (0-7,3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3,6 (0-7,8)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3,4 (0-7,7)</t>
   </si>
   <si>
     <t xml:space="preserve">Condutividade (µS/cm) </t>
@@ -1649,13 +1553,13 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1664,18 +1568,9 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
       <family val="0"/>
     </font>
   </fonts>
@@ -1688,7 +1583,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
@@ -1696,57 +1591,28 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+      <alignment textRotation="0" horizontal="general" vertical="bottom" indent="0"/>
+      <protection hidden="0" locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+      <alignment textRotation="0" horizontal="left" vertical="bottom" indent="0"/>
+      <protection hidden="0" locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+      <alignment textRotation="0" horizontal="left" vertical="bottom" indent="0"/>
+      <protection hidden="0" locked="0"/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
 </styleSheet>
 </file>
 
@@ -1926,14 +1792,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P23"/>
-  <sheetFormatPr defaultColWidth="10.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1983,7 +1849,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>16</v>
       </c>
@@ -2033,7 +1899,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
         <v>32</v>
       </c>
@@ -2083,7 +1949,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>47</v>
       </c>
@@ -2133,7 +1999,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="s">
         <v>63</v>
       </c>
@@ -2183,7 +2049,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" ht="15" customHeight="1">
       <c r="A6" s="1" t="s">
         <v>79</v>
       </c>
@@ -2233,7 +2099,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" ht="15" customHeight="1">
       <c r="A7" s="1" t="s">
         <v>95</v>
       </c>
@@ -2283,7 +2149,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" ht="15" customHeight="1">
       <c r="A8" s="1" t="s">
         <v>109</v>
       </c>
@@ -2333,7 +2199,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" ht="15" customHeight="1">
       <c r="A9" s="1" t="s">
         <v>125</v>
       </c>
@@ -2383,7 +2249,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" ht="15" customHeight="1">
       <c r="A10" s="1" t="s">
         <v>140</v>
       </c>
@@ -2433,7 +2299,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" ht="15" customHeight="1">
       <c r="A11" s="1" t="s">
         <v>156</v>
       </c>
@@ -2483,7 +2349,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" ht="15" customHeight="1">
       <c r="A12" s="1" t="s">
         <v>172</v>
       </c>
@@ -2533,7 +2399,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" ht="15" customHeight="1">
       <c r="A13" s="1" t="s">
         <v>187</v>
       </c>
@@ -2583,7 +2449,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" ht="15" customHeight="1">
       <c r="A14" s="1" t="s">
         <v>201</v>
       </c>
@@ -2633,7 +2499,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" ht="15" customHeight="1">
       <c r="A15" s="1" t="s">
         <v>203</v>
       </c>
@@ -2683,7 +2549,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" ht="15" customHeight="1">
       <c r="A16" s="1" t="s">
         <v>204</v>
       </c>
@@ -2733,7 +2599,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" ht="15" customHeight="1">
       <c r="A17" s="1" t="s">
         <v>210</v>
       </c>
@@ -2783,7 +2649,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" ht="15" customHeight="1">
       <c r="A18" s="1" t="s">
         <v>218</v>
       </c>
@@ -2833,7 +2699,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" ht="15" customHeight="1">
       <c r="A19" s="1" t="s">
         <v>228</v>
       </c>
@@ -2883,7 +2749,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" ht="15" customHeight="1">
       <c r="A20" s="1" t="s">
         <v>243</v>
       </c>
@@ -2933,7 +2799,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" ht="15" customHeight="1">
       <c r="A21" s="1" t="s">
         <v>255</v>
       </c>
@@ -2983,7 +2849,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" ht="15" customHeight="1">
       <c r="A22" s="1" t="s">
         <v>263</v>
       </c>
@@ -3033,7 +2899,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" ht="15" customHeight="1">
       <c r="A23" s="1" t="s">
         <v>267</v>
       </c>
@@ -3084,31 +2950,42 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.7" right="0.7" top="0.597222222222222" bottom="0.597222222222222" header="0.511805555555556" footer="0.511805555555556"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
+  <headerFooter differentOddEven="0" differentFirst="0" scaleWithDoc="0" alignWithMargins="0">
+    <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
+    <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P28"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="23.9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="17.59"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="3" style="2" width="10.66"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="17" style="2" width="11.53"/>
+    <col min="1" max="1" width="23.9" hidden="false" outlineLevel="0" customWidth="1"/>
+    <col min="2" max="2" width="17.59" hidden="false" outlineLevel="0" customWidth="1"/>
+    <col min="3" max="3" width="10.66" hidden="false" outlineLevel="0" customWidth="1"/>
+    <col min="4" max="4" width="10.66" hidden="false" outlineLevel="0" customWidth="1"/>
+    <col min="5" max="5" width="10.66" hidden="false" outlineLevel="0" customWidth="1"/>
+    <col min="6" max="6" width="10.66" hidden="false" outlineLevel="0" customWidth="1"/>
+    <col min="7" max="7" width="10.66" hidden="false" outlineLevel="0" customWidth="1"/>
+    <col min="8" max="8" width="10.66" hidden="false" outlineLevel="0" customWidth="1"/>
+    <col min="9" max="9" width="10.66" hidden="false" outlineLevel="0" customWidth="1"/>
+    <col min="10" max="10" width="10.66" hidden="false" outlineLevel="0" customWidth="1"/>
+    <col min="11" max="11" width="10.66" hidden="false" outlineLevel="0" customWidth="1"/>
+    <col min="12" max="12" width="10.66" hidden="false" outlineLevel="0" customWidth="1"/>
+    <col min="13" max="13" width="10.66" hidden="false" outlineLevel="0" customWidth="1"/>
+    <col min="14" max="14" width="10.66" hidden="false" outlineLevel="0" customWidth="1"/>
+    <col min="15" max="15" width="10.66" hidden="false" outlineLevel="0" customWidth="1"/>
+    <col min="16" max="16" width="10.66" hidden="false" outlineLevel="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" ht="13.5" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>281</v>
       </c>
@@ -3158,7 +3035,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" ht="13.5" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>297</v>
       </c>
@@ -3208,12 +3085,12 @@
         <v>300</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" ht="13.5" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" ht="13.5" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>303</v>
       </c>
@@ -3263,7 +3140,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" ht="13.5" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>319</v>
       </c>
@@ -3304,1055 +3181,956 @@
         <v>331</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>45</v>
+        <v>332</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="6" ht="13.5" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="7" ht="13.5" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>349</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>350</v>
-      </c>
-      <c r="C7" s="3" t="s">
         <v>351</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+    </row>
+    <row r="8" ht="13.5" customHeight="1">
+      <c r="A8" s="2" t="s">
         <v>352</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="B8" s="3" t="s">
         <v>353</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="C8" s="3" t="s">
         <v>354</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="D8" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="E8" s="3" t="s">
         <v>355</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="F8" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G8" s="3" t="s">
         <v>356</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="H8" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="N8" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="O8" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="P8" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="9" ht="13.5" customHeight="1">
+      <c r="A9" s="2" t="s">
         <v>357</v>
       </c>
-      <c r="J7" s="3" t="s">
+      <c r="B9" s="3" t="s">
         <v>358</v>
       </c>
-      <c r="K7" s="2" t="s">
+      <c r="C9" s="3" t="s">
         <v>359</v>
       </c>
-      <c r="L7" s="2" t="s">
+      <c r="D9" s="3" t="s">
         <v>360</v>
       </c>
-      <c r="M7" s="2" t="s">
+      <c r="E9" s="3" t="s">
         <v>361</v>
       </c>
-      <c r="N7" s="2" t="s">
+      <c r="F9" s="3" t="s">
         <v>362</v>
       </c>
-      <c r="O7" s="2" t="s">
+      <c r="G9" s="3" t="s">
         <v>363</v>
       </c>
-      <c r="P7" s="2" t="s">
+      <c r="H9" s="3" t="s">
         <v>364</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="I9" s="3" t="s">
         <v>365</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="J9" s="3" t="s">
         <v>366</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="K9" s="2" t="s">
         <v>367</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="L9" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="M9" s="2" t="s">
         <v>368</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="N9" s="2" t="s">
         <v>369</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="O9" s="2" t="s">
         <v>370</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="P9" s="2" t="s">
         <v>371</v>
       </c>
-      <c r="H8" s="3" t="s">
+    </row>
+    <row r="10" ht="13.5" customHeight="1">
+      <c r="A10" s="2" t="s">
         <v>372</v>
       </c>
-      <c r="I8" s="3" t="s">
+      <c r="B10" s="3" t="s">
         <v>373</v>
       </c>
-      <c r="J8" s="3" t="s">
+      <c r="C10" s="3" t="s">
         <v>374</v>
       </c>
-      <c r="K8" s="2" t="s">
+      <c r="D10" s="3" t="s">
         <v>375</v>
       </c>
-      <c r="L8" s="2" t="s">
+      <c r="E10" s="3" t="s">
         <v>376</v>
       </c>
-      <c r="M8" s="2" t="s">
+      <c r="F10" s="3" t="s">
         <v>377</v>
       </c>
-      <c r="N8" s="2" t="s">
+      <c r="G10" s="3" t="s">
         <v>378</v>
       </c>
-      <c r="O8" s="2" t="s">
+      <c r="H10" s="3" t="s">
         <v>379</v>
       </c>
-      <c r="P8" s="2" t="s">
+      <c r="I10" s="3" t="s">
         <v>380</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="J10" s="3" t="s">
         <v>381</v>
       </c>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-    </row>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="K10" s="2" t="s">
         <v>382</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="L10" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="M10" s="2" t="s">
         <v>383</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="N10" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="O10" s="2" t="s">
         <v>384</v>
       </c>
-      <c r="D10" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="E10" s="3" t="s">
+      <c r="P10" s="2" t="s">
         <v>385</v>
       </c>
-      <c r="F10" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="G10" s="3" t="s">
+    </row>
+    <row r="11" ht="13.5" customHeight="1">
+      <c r="A11" s="2" t="s">
         <v>386</v>
       </c>
-      <c r="H10" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="K10" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="L10" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="M10" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="N10" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="O10" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="P10" s="2" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="B11" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="C11" s="3" t="s">
         <v>388</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="D11" s="3" t="s">
         <v>389</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="E11" s="3" t="s">
         <v>390</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="F11" s="3" t="s">
         <v>391</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="G11" s="3" t="s">
         <v>392</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="H11" s="3" t="s">
         <v>393</v>
       </c>
-      <c r="H11" s="3" t="s">
+      <c r="I11" s="3" t="s">
         <v>394</v>
       </c>
-      <c r="I11" s="3" t="s">
+      <c r="J11" s="3" t="s">
         <v>395</v>
       </c>
-      <c r="J11" s="3" t="s">
+      <c r="K11" s="2" t="s">
         <v>396</v>
       </c>
-      <c r="K11" s="2" t="s">
+      <c r="L11" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="M11" s="2" t="s">
         <v>397</v>
       </c>
-      <c r="L11" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="M11" s="2" t="s">
+      <c r="N11" s="2" t="s">
         <v>398</v>
       </c>
-      <c r="N11" s="2" t="s">
+      <c r="O11" s="2" t="s">
         <v>399</v>
       </c>
-      <c r="O11" s="2" t="s">
+      <c r="P11" s="2" t="s">
         <v>400</v>
       </c>
-      <c r="P11" s="2" t="s">
+    </row>
+    <row r="12" ht="13.5" customHeight="1">
+      <c r="A12" s="2" t="s">
         <v>401</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+      <c r="B12" s="3" t="s">
         <v>402</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="C12" s="3" t="s">
         <v>403</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="D12" s="3" t="s">
         <v>404</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="E12" s="3" t="s">
         <v>405</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="F12" s="3" t="s">
         <v>406</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="G12" s="3" t="s">
         <v>407</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="H12" s="3" t="s">
         <v>408</v>
       </c>
-      <c r="H12" s="3" t="s">
+      <c r="I12" s="3" t="s">
         <v>409</v>
       </c>
-      <c r="I12" s="3" t="s">
+      <c r="J12" s="3" t="s">
         <v>410</v>
       </c>
-      <c r="J12" s="3" t="s">
+      <c r="K12" s="2" t="s">
         <v>411</v>
       </c>
-      <c r="K12" s="2" t="s">
+      <c r="L12" s="2" t="s">
         <v>412</v>
-      </c>
-      <c r="L12" s="2" t="s">
-        <v>136</v>
       </c>
       <c r="M12" s="2" t="s">
         <v>413</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>136</v>
+        <v>414</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="P12" s="2" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="13" ht="13.5" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>416</v>
-      </c>
-      <c r="B13" s="3" t="s">
         <v>417</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
+    </row>
+    <row r="14" ht="13.5" customHeight="1">
+      <c r="A14" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="B14" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E14" s="3" t="s">
         <v>419</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="F14" s="3" t="s">
         <v>420</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="G14" s="3" t="s">
         <v>421</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="H14" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="I14" s="3" t="s">
         <v>422</v>
       </c>
-      <c r="H13" s="3" t="s">
+      <c r="J14" s="3" t="s">
         <v>423</v>
       </c>
-      <c r="I13" s="3" t="s">
+      <c r="K14" s="2" t="s">
         <v>424</v>
       </c>
-      <c r="J13" s="3" t="s">
+      <c r="L14" s="2" t="s">
         <v>425</v>
       </c>
-      <c r="K13" s="2" t="s">
+      <c r="M14" s="2" t="s">
         <v>426</v>
       </c>
-      <c r="L13" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="M13" s="2" t="s">
+      <c r="N14" s="2" t="s">
         <v>427</v>
       </c>
-      <c r="N13" s="2" t="s">
+      <c r="O14" s="2" t="s">
         <v>428</v>
       </c>
-      <c r="O13" s="2" t="s">
+      <c r="P14" s="2" t="s">
         <v>429</v>
       </c>
-      <c r="P13" s="2" t="s">
+    </row>
+    <row r="15" ht="13.5" customHeight="1">
+      <c r="A15" s="2" t="s">
         <v>430</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+      <c r="B15" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="E15" s="3" t="s">
         <v>431</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="F15" s="3" t="s">
         <v>432</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="G15" s="3" t="s">
         <v>433</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="H15" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="I15" s="3" t="s">
         <v>434</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="J15" s="3" t="s">
         <v>435</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="K15" s="2" t="s">
         <v>436</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="L15" s="2" t="s">
         <v>437</v>
       </c>
-      <c r="H14" s="3" t="s">
+      <c r="M15" s="2" t="s">
         <v>438</v>
       </c>
-      <c r="I14" s="3" t="s">
+      <c r="N15" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="O15" s="2" t="s">
         <v>439</v>
       </c>
-      <c r="J14" s="3" t="s">
+      <c r="P15" s="2" t="s">
         <v>440</v>
       </c>
-      <c r="K14" s="2" t="s">
+    </row>
+    <row r="16" ht="13.5" customHeight="1">
+      <c r="A16" s="2" t="s">
         <v>441</v>
       </c>
-      <c r="L14" s="2" t="s">
+      <c r="B16" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>438</v>
+      </c>
+      <c r="K16" s="2" t="s">
         <v>442</v>
       </c>
-      <c r="M14" s="2" t="s">
+      <c r="L16" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="N16" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="O16" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="P16" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="17" ht="13.5" customHeight="1">
+      <c r="A17" s="2" t="s">
         <v>443</v>
       </c>
-      <c r="N14" s="2" t="s">
+      <c r="B17" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="M17" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="N17" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="O17" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="P17" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="18" ht="13.5" customHeight="1">
+      <c r="A18" s="2" t="s">
         <v>444</v>
       </c>
-      <c r="O14" s="2" t="s">
+    </row>
+    <row r="19" ht="13.5" customHeight="1">
+      <c r="A19" s="2" t="s">
         <v>445</v>
       </c>
-      <c r="P14" s="2" t="s">
+      <c r="B19" s="2" t="s">
         <v>446</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
+      <c r="C19" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="E19" s="2" t="s">
         <v>447</v>
       </c>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
-    </row>
-    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
+      <c r="F19" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="L19" s="2" t="s">
         <v>448</v>
       </c>
-      <c r="B16" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E16" s="3" t="s">
+      <c r="M19" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="N19" s="2" t="s">
         <v>449</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="O19" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="P19" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="20" ht="13.5" customHeight="1">
+      <c r="A20" s="2" t="s">
         <v>450</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="B20" s="2" t="s">
         <v>451</v>
       </c>
-      <c r="H16" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="I16" s="3" t="s">
+      <c r="C20" s="2" t="s">
         <v>452</v>
       </c>
-      <c r="J16" s="3" t="s">
+      <c r="D20" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>453</v>
       </c>
-      <c r="K16" s="2" t="s">
+      <c r="F20" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="G20" s="2" t="s">
         <v>454</v>
       </c>
-      <c r="L16" s="2" t="s">
+      <c r="H20" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="L20" s="2" t="s">
         <v>455</v>
       </c>
-      <c r="M16" s="2" t="s">
+      <c r="M20" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="N20" s="2" t="s">
         <v>456</v>
       </c>
-      <c r="N16" s="2" t="s">
+      <c r="O20" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="P20" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="21" ht="13.5" customHeight="1">
+      <c r="A21" s="2" t="s">
         <v>457</v>
       </c>
-      <c r="O16" s="2" t="s">
+      <c r="B21" s="2" t="s">
         <v>458</v>
       </c>
-      <c r="P16" s="2" t="s">
+      <c r="C21" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>459</v>
       </c>
-    </row>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
+      <c r="E21" s="2" t="s">
+        <v>459</v>
+      </c>
+      <c r="F21" s="2" t="s">
         <v>460</v>
       </c>
-      <c r="B17" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="D17" s="3" t="s">
+      <c r="G21" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="H21" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="I21" s="2" t="s">
         <v>461</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="J21" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="L21" s="2" t="s">
         <v>462</v>
       </c>
-      <c r="G17" s="3" t="s">
+      <c r="M21" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="N21" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="O21" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="P21" s="2" t="s">
         <v>463</v>
       </c>
-      <c r="H17" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="I17" s="3" t="s">
+    </row>
+    <row r="22" ht="13.5" customHeight="1">
+      <c r="A22" s="2" t="s">
         <v>464</v>
       </c>
-      <c r="J17" s="3" t="s">
+      <c r="B22" s="2" t="s">
         <v>465</v>
       </c>
-      <c r="K17" s="2" t="s">
+      <c r="C22" s="2" t="s">
         <v>466</v>
       </c>
-      <c r="L17" s="2" t="s">
+      <c r="D22" s="2" t="s">
         <v>467</v>
       </c>
-      <c r="M17" s="2" t="s">
+      <c r="E22" s="2" t="s">
         <v>468</v>
       </c>
-      <c r="N17" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="O17" s="2" t="s">
+      <c r="F22" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="H22" s="2" t="s">
         <v>469</v>
       </c>
-      <c r="P17" s="2" t="s">
+      <c r="I22" s="2" t="s">
         <v>470</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
+      <c r="J22" s="2" t="s">
         <v>471</v>
       </c>
-      <c r="B18" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="J18" s="3" t="s">
-        <v>468</v>
-      </c>
-      <c r="K18" s="2" t="s">
+      <c r="K22" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="L22" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="M22" s="2" t="s">
         <v>472</v>
       </c>
-      <c r="L18" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="M18" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="N18" s="2" t="s">
-        <v>472</v>
-      </c>
-      <c r="O18" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="P18" s="2" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
+      <c r="N22" s="2" t="s">
         <v>473</v>
       </c>
-      <c r="B19" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="I19" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="J19" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="K19" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="L19" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="M19" s="2" t="s">
-        <v>472</v>
-      </c>
-      <c r="N19" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="O19" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="P19" s="2" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
+      <c r="O22" s="2" t="s">
         <v>474</v>
       </c>
-    </row>
-    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2" t="s">
+      <c r="P22" s="2" t="s">
         <v>475</v>
       </c>
-      <c r="B21" s="2" t="s">
+    </row>
+    <row r="23" ht="13.5" customHeight="1">
+      <c r="A23" s="2" t="s">
         <v>476</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="E21" s="2" t="s">
+      <c r="B23" s="2" t="s">
         <v>477</v>
       </c>
-      <c r="F21" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="I21" s="2" t="s">
-        <v>468</v>
-      </c>
-      <c r="J21" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="K21" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="L21" s="2" t="s">
+      <c r="C23" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>478</v>
       </c>
-      <c r="M21" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="N21" s="2" t="s">
+      <c r="E23" s="2" t="s">
         <v>479</v>
       </c>
-      <c r="O21" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="P21" s="2" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
+      <c r="F23" s="2" t="s">
         <v>480</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="G23" s="2" t="s">
         <v>481</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>482</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>483</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>484</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="I22" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="J22" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="K22" s="2" t="s">
-        <v>468</v>
-      </c>
-      <c r="L22" s="2" t="s">
-        <v>485</v>
-      </c>
-      <c r="M22" s="2" t="s">
-        <v>476</v>
-      </c>
-      <c r="N22" s="2" t="s">
-        <v>486</v>
-      </c>
-      <c r="O22" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="P22" s="2" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
-        <v>487</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>488</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>482</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>489</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>489</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>490</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>188</v>
       </c>
       <c r="H23" s="2" t="s">
         <v>458</v>
       </c>
       <c r="I23" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="J23" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="L23" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="M23" s="2" t="s">
+        <v>483</v>
+      </c>
+      <c r="N23" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="O23" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="P23" s="2" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="24" ht="13.5" customHeight="1">
+      <c r="A24" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>488</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>489</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>459</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="J24" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="K24" s="2" t="s">
         <v>491</v>
       </c>
-      <c r="J23" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="K23" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="L23" s="2" t="s">
+      <c r="L24" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="M24" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="N24" s="2" t="s">
         <v>492</v>
       </c>
-      <c r="M23" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="N23" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="O23" s="2" t="s">
-        <v>468</v>
-      </c>
-      <c r="P23" s="2" t="s">
+      <c r="O24" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="P24" s="2" t="s">
         <v>493</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
+    <row r="25" ht="13.5" customHeight="1">
+      <c r="A25" s="2" t="s">
         <v>494</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B25" s="2" t="s">
+        <v>483</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>495</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="D25" s="2" t="s">
         <v>496</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="E25" s="2" t="s">
         <v>497</v>
       </c>
-      <c r="E24" s="2" t="s">
+      <c r="F25" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="J25" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="L25" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="M25" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="N25" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="O25" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="P25" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="26" ht="13.5" customHeight="1">
+      <c r="A26" s="2" t="s">
         <v>498</v>
       </c>
-      <c r="F24" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="H24" s="2" t="s">
+      <c r="B26" s="2" t="s">
         <v>499</v>
       </c>
-      <c r="I24" s="2" t="s">
+      <c r="C26" s="2" t="s">
         <v>500</v>
       </c>
-      <c r="J24" s="2" t="s">
+      <c r="D26" s="2" t="s">
         <v>501</v>
       </c>
-      <c r="K24" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="L24" s="2" t="s">
-        <v>468</v>
-      </c>
-      <c r="M24" s="2" t="s">
+      <c r="E26" s="2" t="s">
         <v>502</v>
       </c>
-      <c r="N24" s="2" t="s">
+      <c r="F26" s="2" t="s">
         <v>503</v>
       </c>
-      <c r="O24" s="2" t="s">
+      <c r="G26" s="2" t="s">
         <v>504</v>
       </c>
-      <c r="P24" s="2" t="s">
+      <c r="H26" s="2" t="s">
         <v>505</v>
       </c>
-    </row>
-    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
+      <c r="I26" s="2" t="s">
         <v>506</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="J26" s="2" t="s">
         <v>507</v>
       </c>
-      <c r="C25" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="D25" s="2" t="s">
+      <c r="K26" s="2" t="s">
         <v>508</v>
       </c>
-      <c r="E25" s="2" t="s">
+      <c r="L26" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="M26" s="2" t="s">
         <v>509</v>
       </c>
-      <c r="F25" s="2" t="s">
+      <c r="N26" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="O26" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="P26" s="2" t="s">
         <v>510</v>
       </c>
-      <c r="G25" s="2" t="s">
-        <v>511</v>
-      </c>
-      <c r="H25" s="2" t="s">
-        <v>488</v>
-      </c>
-      <c r="I25" s="2" t="s">
-        <v>512</v>
-      </c>
-      <c r="J25" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="K25" s="2" t="s">
-        <v>507</v>
-      </c>
-      <c r="L25" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="M25" s="2" t="s">
-        <v>513</v>
-      </c>
-      <c r="N25" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="O25" s="2" t="s">
-        <v>514</v>
-      </c>
-      <c r="P25" s="2" t="s">
-        <v>515</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
-        <v>516</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>517</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>518</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>486</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>519</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>481</v>
-      </c>
-      <c r="H26" s="2" t="s">
-        <v>489</v>
-      </c>
-      <c r="I26" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="J26" s="2" t="s">
-        <v>520</v>
-      </c>
-      <c r="K26" s="2" t="s">
-        <v>521</v>
-      </c>
-      <c r="L26" s="2" t="s">
-        <v>468</v>
-      </c>
-      <c r="M26" s="2" t="s">
-        <v>517</v>
-      </c>
-      <c r="N26" s="2" t="s">
-        <v>522</v>
-      </c>
-      <c r="O26" s="2" t="s">
-        <v>488</v>
-      </c>
-      <c r="P26" s="2" t="s">
-        <v>523</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="2" t="s">
-        <v>524</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>513</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>525</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>526</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>527</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>468</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>468</v>
-      </c>
-      <c r="I27" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="J27" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="K27" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="L27" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="M27" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="N27" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="O27" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="P27" s="2" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="s">
-        <v>528</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>529</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>530</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>531</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>532</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>533</v>
-      </c>
-      <c r="G28" s="2" t="s">
-        <v>534</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>535</v>
-      </c>
-      <c r="I28" s="2" t="s">
-        <v>536</v>
-      </c>
-      <c r="J28" s="2" t="s">
-        <v>537</v>
-      </c>
-      <c r="K28" s="2" t="s">
-        <v>538</v>
-      </c>
-      <c r="L28" s="2" t="s">
-        <v>486</v>
-      </c>
-      <c r="M28" s="2" t="s">
-        <v>539</v>
-      </c>
-      <c r="N28" s="2" t="s">
-        <v>279</v>
-      </c>
-      <c r="O28" s="2" t="s">
-        <v>479</v>
-      </c>
-      <c r="P28" s="2" t="s">
-        <v>540</v>
-      </c>
-    </row>
+    </row>
+    <row r="1048575" ht="12.8" customHeight="1"/>
+    <row r="1048576" ht="12.8" customHeight="1"/>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;KffffffPágina &amp;P</oddFooter>
+  <headerFooter differentOddEven="0" differentFirst="0" scaleWithDoc="0" alignWithMargins="0">
+    <oddHeader>&amp;L&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;Kffffff&amp;A&amp;R</oddHeader>
+    <oddFooter>&amp;L&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;KffffffPágina &amp;P&amp;R</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>